<commit_message>
save Fri, Oct 23, 2020 11:14:43 PM
</commit_message>
<xml_diff>
--- a/output/dipole_values.xlsx
+++ b/output/dipole_values.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eligh\summer\research\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F7A0C7E-C291-4948-96F5-8F283B72806A}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A4D8A93-12BD-4989-BBDE-8D5FD3F72E7B}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{427F2F01-03BB-4629-B369-0F23A242E73E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{427F2F01-03BB-4629-B369-0F23A242E73E}"/>
   </bookViews>
   <sheets>
-    <sheet name="wB97X-2(TQZ)" sheetId="1" r:id="rId1"/>
+    <sheet name="wB97X-2TQZ" sheetId="1" r:id="rId1"/>
     <sheet name="WFT" sheetId="13" r:id="rId2"/>
     <sheet name="B2PLYP" sheetId="2" r:id="rId3"/>
     <sheet name="B2GPPLYP" sheetId="3" r:id="rId4"/>

</xml_diff>

<commit_message>
save Tue, Oct 27, 2020 11:07:38 PM
</commit_message>
<xml_diff>
--- a/output/dipole_values.xlsx
+++ b/output/dipole_values.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eligh\summer\research\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A4D8A93-12BD-4989-BBDE-8D5FD3F72E7B}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE66D11E-4C3D-44CE-87C6-800618AC047B}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{427F2F01-03BB-4629-B369-0F23A242E73E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="9" xr2:uid="{427F2F01-03BB-4629-B369-0F23A242E73E}"/>
   </bookViews>
   <sheets>
     <sheet name="wB97X-2TQZ" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
     <sheet name="DSD-PBEP86" sheetId="6" r:id="rId7"/>
     <sheet name="PWPB95-D3" sheetId="7" r:id="rId8"/>
     <sheet name="XYG3" sheetId="8" r:id="rId9"/>
-    <sheet name="XYGJ-OS" sheetId="9" r:id="rId10"/>
+    <sheet name="XYGJOS" sheetId="9" r:id="rId10"/>
     <sheet name="RMP2_5Z" sheetId="10" r:id="rId11"/>
     <sheet name="RMP2_QZ" sheetId="11" r:id="rId12"/>
     <sheet name="RMP2_TZ" sheetId="12" r:id="rId13"/>

</xml_diff>

<commit_message>
save Mon, Nov 16, 2020  2:43:15 AM
</commit_message>
<xml_diff>
--- a/output/dipole_values.xlsx
+++ b/output/dipole_values.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eligh\summer\research\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE66D11E-4C3D-44CE-87C6-800618AC047B}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41B59E78-974F-45A8-9493-3C60F101B0DD}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="9" xr2:uid="{427F2F01-03BB-4629-B369-0F23A242E73E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="10" xr2:uid="{427F2F01-03BB-4629-B369-0F23A242E73E}"/>
   </bookViews>
   <sheets>
     <sheet name="wB97X-2TQZ" sheetId="1" r:id="rId1"/>
@@ -23,9 +23,10 @@
     <sheet name="PWPB95-D3" sheetId="7" r:id="rId8"/>
     <sheet name="XYG3" sheetId="8" r:id="rId9"/>
     <sheet name="XYGJOS" sheetId="9" r:id="rId10"/>
-    <sheet name="RMP2_5Z" sheetId="10" r:id="rId11"/>
-    <sheet name="RMP2_QZ" sheetId="11" r:id="rId12"/>
-    <sheet name="RMP2_TZ" sheetId="12" r:id="rId13"/>
+    <sheet name="wB97M2" sheetId="14" r:id="rId11"/>
+    <sheet name="RMP2_5Z" sheetId="10" r:id="rId12"/>
+    <sheet name="RMP2_QZ" sheetId="11" r:id="rId13"/>
+    <sheet name="RMP2_TZ" sheetId="12" r:id="rId14"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -45,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1819" uniqueCount="186">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1988" uniqueCount="188">
   <si>
     <t>wB97X-2</t>
   </si>
@@ -604,6 +605,12 @@
   <si>
     <t>CH2-trip</t>
   </si>
+  <si>
+    <t>wB97M2</t>
+  </si>
+  <si>
+    <t>SiH3</t>
+  </si>
 </sst>
 </file>
 
@@ -970,7 +977,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E753B392-0225-4F96-9A7E-DEB3BFF53393}">
-  <dimension ref="A1:G153"/>
+  <dimension ref="A1:G154"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -4490,6 +4497,26 @@
       </c>
       <c r="G153">
         <v>1.4129</v>
+      </c>
+    </row>
+    <row r="154" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A154" t="s">
+        <v>187</v>
+      </c>
+      <c r="B154">
+        <v>8.3999999999999995E-3</v>
+      </c>
+      <c r="C154">
+        <v>8.3000000000000001E-3</v>
+      </c>
+      <c r="D154">
+        <v>4.5113049159043003E-2</v>
+      </c>
+      <c r="E154">
+        <v>8.5000000000000006E-3</v>
+      </c>
+      <c r="F154">
+        <v>4.6256761180151797E-2</v>
       </c>
     </row>
   </sheetData>
@@ -4499,7 +4526,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E7015F87-6BC2-4AB3-BAE2-878DAC4C553C}">
-  <dimension ref="A1:G153"/>
+  <dimension ref="A1:G154"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -8019,6 +8046,26 @@
       </c>
       <c r="G153">
         <v>1.6126</v>
+      </c>
+    </row>
+    <row r="154" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A154" t="s">
+        <v>187</v>
+      </c>
+      <c r="B154">
+        <v>1.2834980346062499E-2</v>
+      </c>
+      <c r="C154">
+        <v>1.2834980346062499E-2</v>
+      </c>
+      <c r="D154">
+        <v>1.6093285867857E-2</v>
+      </c>
+      <c r="E154">
+        <v>1.0420479357469901E-2</v>
+      </c>
+      <c r="F154">
+        <v>1.5717131778708902E-2</v>
       </c>
     </row>
   </sheetData>
@@ -8027,6 +8074,1840 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F16311FB-254B-441A-B73D-24711CD7F8B9}">
+  <dimension ref="A1:G154"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2">
+        <v>1.5191025173620401</v>
+      </c>
+      <c r="C2">
+        <v>1.5424405782726101</v>
+      </c>
+      <c r="D2">
+        <v>1.4948304254732101</v>
+      </c>
+      <c r="E2">
+        <v>1.5276000000000001</v>
+      </c>
+      <c r="F2">
+        <v>1.4978803220290899</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3">
+        <v>0.51759281844650096</v>
+      </c>
+      <c r="C3">
+        <v>0.51416168491143599</v>
+      </c>
+      <c r="D3">
+        <v>0.502470415864122</v>
+      </c>
+      <c r="E3">
+        <v>0.51225549965430905</v>
+      </c>
+      <c r="F3">
+        <v>0.50310581107022401</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4">
+        <v>0.37221442804932098</v>
+      </c>
+      <c r="C4">
+        <v>0.36306473914920301</v>
+      </c>
+      <c r="D4">
+        <v>0.339936358830012</v>
+      </c>
+      <c r="E4">
+        <v>0.35499999999999998</v>
+      </c>
+      <c r="F4">
+        <v>0.333709487214297</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5">
+        <v>0.85600422922431396</v>
+      </c>
+      <c r="C5">
+        <v>0.85600422922431396</v>
+      </c>
+      <c r="D5">
+        <v>0.95652372814759301</v>
+      </c>
+      <c r="E5">
+        <v>0.85536000000000001</v>
+      </c>
+      <c r="F5">
+        <v>0.95639664903413701</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7">
+        <v>0.50895144568417705</v>
+      </c>
+      <c r="C7">
+        <v>0.53265930621354096</v>
+      </c>
+      <c r="D7">
+        <v>0.50844312959153104</v>
+      </c>
+      <c r="E7">
+        <v>0.51100000000000001</v>
+      </c>
+      <c r="F7">
+        <v>0.50996807777917297</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8">
+        <v>0.76552397195695399</v>
+      </c>
+      <c r="C8">
+        <v>0.766921841482615</v>
+      </c>
+      <c r="D8">
+        <v>0.61951018689544202</v>
+      </c>
+      <c r="E8">
+        <v>0.77403826605729698</v>
+      </c>
+      <c r="F8">
+        <v>0.61582489477228397</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9">
+        <v>0.885994876162158</v>
+      </c>
+      <c r="C9">
+        <v>0.88840937733134095</v>
+      </c>
+      <c r="D9">
+        <v>0.74798706856657304</v>
+      </c>
+      <c r="E9">
+        <v>0.88849999999999996</v>
+      </c>
+      <c r="F9">
+        <v>0.74392054000599594</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11">
+        <v>1.00595746391353</v>
+      </c>
+      <c r="C11">
+        <v>1.00659285911963</v>
+      </c>
+      <c r="D11">
+        <v>0.88929893058376597</v>
+      </c>
+      <c r="E11">
+        <v>1.0077</v>
+      </c>
+      <c r="F11">
+        <v>0.88739274532663903</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>18</v>
+      </c>
+      <c r="B13">
+        <v>2.7590124435023999</v>
+      </c>
+      <c r="C13">
+        <v>2.75964783852791</v>
+      </c>
+      <c r="D13">
+        <v>2.3439723883497599</v>
+      </c>
+      <c r="E13">
+        <v>2.7597</v>
+      </c>
+      <c r="F13">
+        <v>2.3435911513705698</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>19</v>
+      </c>
+      <c r="B14">
+        <v>1.2470263507150401</v>
+      </c>
+      <c r="C14">
+        <v>1.2447389288399</v>
+      </c>
+      <c r="D14">
+        <v>0.87811597762909799</v>
+      </c>
+      <c r="E14">
+        <v>1.2543</v>
+      </c>
+      <c r="F14">
+        <v>0.88116587418497305</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>20</v>
+      </c>
+      <c r="B15">
+        <v>0.75472225616206501</v>
+      </c>
+      <c r="C15">
+        <v>0.75535765118757703</v>
+      </c>
+      <c r="D15">
+        <v>0.77403826605729698</v>
+      </c>
+      <c r="E15">
+        <v>0.75670000000000004</v>
+      </c>
+      <c r="F15">
+        <v>0.77416534499016298</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>26</v>
+      </c>
+      <c r="B21">
+        <v>0.799454068522509</v>
+      </c>
+      <c r="C21">
+        <v>0.79907283154331998</v>
+      </c>
+      <c r="D21">
+        <v>0.68038103366237601</v>
+      </c>
+      <c r="E21">
+        <v>0.68456955808518805</v>
+      </c>
+      <c r="F21">
+        <v>0.68012687561605301</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>169</v>
+      </c>
+      <c r="B26">
+        <v>1.83108149321846</v>
+      </c>
+      <c r="C26">
+        <v>1.82942946609795</v>
+      </c>
+      <c r="D26">
+        <v>1.7852059696495599</v>
+      </c>
+      <c r="E26">
+        <v>1.83120857224162</v>
+      </c>
+      <c r="F26">
+        <v>1.7844434955106001</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>31</v>
+      </c>
+      <c r="B27">
+        <v>0.60947094469775098</v>
+      </c>
+      <c r="C27">
+        <v>0.62838157253167204</v>
+      </c>
+      <c r="D27">
+        <v>0.61086881377193702</v>
+      </c>
+      <c r="E27">
+        <v>0.61109999999999998</v>
+      </c>
+      <c r="F27">
+        <v>0.61125005075112704</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>34</v>
+      </c>
+      <c r="B30">
+        <v>1.94621507890236</v>
+      </c>
+      <c r="C30">
+        <v>1.94519844671707</v>
+      </c>
+      <c r="D30">
+        <v>1.86920519682598</v>
+      </c>
+      <c r="E30">
+        <v>1.9534499999999999</v>
+      </c>
+      <c r="F30">
+        <v>1.8681885653630499</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>35</v>
+      </c>
+      <c r="B31">
+        <v>1.8500162658636199</v>
+      </c>
+      <c r="C31">
+        <v>1.8497621079978901</v>
+      </c>
+      <c r="D31">
+        <v>1.7661441174394701</v>
+      </c>
+      <c r="E31">
+        <v>1.8520495302341999</v>
+      </c>
+      <c r="F31">
+        <v>1.76411085343007</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>36</v>
+      </c>
+      <c r="B32">
+        <v>5.8616465373710502</v>
+      </c>
+      <c r="C32">
+        <v>5.8617736163942098</v>
+      </c>
+      <c r="D32">
+        <v>5.7644310926887901</v>
+      </c>
+      <c r="E32">
+        <v>5.8593591151347297</v>
+      </c>
+      <c r="F32">
+        <v>5.76227074947563</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>41</v>
+      </c>
+      <c r="B37">
+        <v>3.0192702612662701</v>
+      </c>
+      <c r="C37">
+        <v>3.0192702612662701</v>
+      </c>
+      <c r="D37">
+        <v>2.9149383929122701</v>
+      </c>
+      <c r="E37">
+        <v>3.0131999999999999</v>
+      </c>
+      <c r="F37">
+        <v>2.91709873495159</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>42</v>
+      </c>
+      <c r="B38">
+        <v>0.99032674523851105</v>
+      </c>
+      <c r="C38">
+        <v>0.99058090346542504</v>
+      </c>
+      <c r="D38">
+        <v>0.88485116486340998</v>
+      </c>
+      <c r="E38">
+        <v>0.99172400000000005</v>
+      </c>
+      <c r="F38">
+        <v>0.88840937715075097</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>44</v>
+      </c>
+      <c r="B40">
+        <v>2.0147106665172099</v>
+      </c>
+      <c r="C40">
+        <v>2.0125503232137598</v>
+      </c>
+      <c r="D40">
+        <v>1.27002765255284</v>
+      </c>
+      <c r="E40">
+        <v>2.0130499999999998</v>
+      </c>
+      <c r="F40">
+        <v>1.2726963115877501</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>45</v>
+      </c>
+      <c r="B41">
+        <v>8.9209466855154795E-2</v>
+      </c>
+      <c r="C41">
+        <v>7.7391118694384003E-2</v>
+      </c>
+      <c r="D41">
+        <v>0.165075637452191</v>
+      </c>
+      <c r="E41">
+        <v>9.1369000000000006E-2</v>
+      </c>
+      <c r="F41">
+        <v>0.151605262080616</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>46</v>
+      </c>
+      <c r="B42">
+        <v>1.80388658451928</v>
+      </c>
+      <c r="C42">
+        <v>1.80401366363274</v>
+      </c>
+      <c r="D42">
+        <v>2.01089829564178</v>
+      </c>
+      <c r="E42">
+        <v>1.7932110000000001</v>
+      </c>
+      <c r="F42">
+        <v>2.0051797405927601</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>47</v>
+      </c>
+      <c r="B43">
+        <v>0.79335427613311904</v>
+      </c>
+      <c r="C43">
+        <v>0.79348135452421498</v>
+      </c>
+      <c r="D43">
+        <v>0.69372432992049404</v>
+      </c>
+      <c r="E43">
+        <v>0.78306087000000002</v>
+      </c>
+      <c r="F43">
+        <v>0.68533711493360805</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>48</v>
+      </c>
+      <c r="B44">
+        <v>2.2870409906687601</v>
+      </c>
+      <c r="C44">
+        <v>2.2848806475458998</v>
+      </c>
+      <c r="D44">
+        <v>2.2553983163395301</v>
+      </c>
+      <c r="E44">
+        <v>2.2846264000000001</v>
+      </c>
+      <c r="F44">
+        <v>2.2587023707611298</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>54</v>
+      </c>
+      <c r="B50">
+        <v>2.4828697490171798</v>
+      </c>
+      <c r="C50">
+        <v>2.4817260380796098</v>
+      </c>
+      <c r="D50">
+        <v>2.5065064455193098</v>
+      </c>
+      <c r="E50">
+        <v>2.4838863799999999</v>
+      </c>
+      <c r="F50">
+        <v>2.50548981333402</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>55</v>
+      </c>
+      <c r="B51">
+        <v>1.91279329824886</v>
+      </c>
+      <c r="C51">
+        <v>1.91114127121865</v>
+      </c>
+      <c r="D51">
+        <v>1.83972286616138</v>
+      </c>
+      <c r="E51">
+        <v>1.9105058699999999</v>
+      </c>
+      <c r="F51">
+        <v>1.83641881173977</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>65</v>
+      </c>
+      <c r="B61">
+        <v>3.05104001452837</v>
+      </c>
+      <c r="C61">
+        <v>3.0510400147089598</v>
+      </c>
+      <c r="D61">
+        <v>2.71161197192645</v>
+      </c>
+      <c r="E61">
+        <v>3.0515479999999999</v>
+      </c>
+      <c r="F61">
+        <v>2.71008702364851</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>66</v>
+      </c>
+      <c r="B62">
+        <v>1.71124598376788</v>
+      </c>
+      <c r="C62">
+        <v>1.7099751940780401</v>
+      </c>
+      <c r="D62">
+        <v>1.41083119865797</v>
+      </c>
+      <c r="E62">
+        <v>1.7217935</v>
+      </c>
+      <c r="F62">
+        <v>1.4146435684498699</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>67</v>
+      </c>
+      <c r="B63">
+        <v>0.49713309743311102</v>
+      </c>
+      <c r="C63">
+        <v>0.49586230774326601</v>
+      </c>
+      <c r="D63">
+        <v>0.43524561830029501</v>
+      </c>
+      <c r="E63">
+        <v>0.50285164999999998</v>
+      </c>
+      <c r="F63">
+        <v>0.43156032834421898</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>68</v>
+      </c>
+      <c r="B64">
+        <v>0.78814403645438402</v>
+      </c>
+      <c r="C64">
+        <v>0.78916066827849596</v>
+      </c>
+      <c r="D64">
+        <v>0.66233581381816897</v>
+      </c>
+      <c r="E64">
+        <v>0.7919564</v>
+      </c>
+      <c r="F64">
+        <v>0.65992131246839603</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>69</v>
+      </c>
+      <c r="B65">
+        <v>2.6129986580797002</v>
+      </c>
+      <c r="C65">
+        <v>2.6025781789028199</v>
+      </c>
+      <c r="D65">
+        <v>2.3813336179086102</v>
+      </c>
+      <c r="E65">
+        <v>2.6151590012025601</v>
+      </c>
+      <c r="F65">
+        <v>2.3884500426638802</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>70</v>
+      </c>
+      <c r="B66">
+        <v>1.89690842188869</v>
+      </c>
+      <c r="C66">
+        <v>1.89576471058994</v>
+      </c>
+      <c r="D66">
+        <v>1.7417449471595501</v>
+      </c>
+      <c r="E66">
+        <v>1.9070747422900001</v>
+      </c>
+      <c r="F66">
+        <v>1.74504900121998</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>71</v>
+      </c>
+      <c r="B67">
+        <v>1.1292241064477</v>
+      </c>
+      <c r="C67">
+        <v>1.09744037496709</v>
+      </c>
+      <c r="D67">
+        <v>1.0932607455115599</v>
+      </c>
+      <c r="E67">
+        <v>1.135578057</v>
+      </c>
+      <c r="F67">
+        <v>1.0951669314910499</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>73</v>
+      </c>
+      <c r="B69">
+        <v>3.14876377530328</v>
+      </c>
+      <c r="C69">
+        <v>3.1474929852522502</v>
+      </c>
+      <c r="D69">
+        <v>3.0299448984894699</v>
+      </c>
+      <c r="E69">
+        <v>3.1500345655339999</v>
+      </c>
+      <c r="F69">
+        <v>3.0313427676539502</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>79</v>
+      </c>
+      <c r="B75">
+        <v>0.27156785019317498</v>
+      </c>
+      <c r="C75">
+        <v>0.27245740326501</v>
+      </c>
+      <c r="D75">
+        <v>0.34425704530147</v>
+      </c>
+      <c r="E75">
+        <v>0.243865895762681</v>
+      </c>
+      <c r="F75">
+        <v>0.35264426028835599</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>80</v>
+      </c>
+      <c r="B76">
+        <v>1.84785592292135</v>
+      </c>
+      <c r="C76">
+        <v>1.84772884380789</v>
+      </c>
+      <c r="D76">
+        <v>1.78012280908429</v>
+      </c>
+      <c r="E76">
+        <v>1.84849131812</v>
+      </c>
+      <c r="F76">
+        <v>1.7783437029406199</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>83</v>
+      </c>
+      <c r="B79">
+        <v>2.9104906266501498</v>
+      </c>
+      <c r="C79">
+        <v>2.9107447846964698</v>
+      </c>
+      <c r="D79">
+        <v>3.08128481969313</v>
+      </c>
+      <c r="E79">
+        <v>2.9120155747399998</v>
+      </c>
+      <c r="F79">
+        <v>3.0810306616468099</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>94</v>
+      </c>
+      <c r="B90">
+        <v>6.1300374119851897</v>
+      </c>
+      <c r="C90">
+        <v>6.1294020169596797</v>
+      </c>
+      <c r="D90">
+        <v>6.0912783131715598</v>
+      </c>
+      <c r="E90">
+        <v>6.1311811230000002</v>
+      </c>
+      <c r="F90">
+        <v>6.0954719206650099</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>95</v>
+      </c>
+      <c r="B91">
+        <v>7.1387906142276902</v>
+      </c>
+      <c r="C91">
+        <v>7.1401884837533496</v>
+      </c>
+      <c r="D91">
+        <v>7.04551461863137</v>
+      </c>
+      <c r="E91">
+        <v>7.1478132240000001</v>
+      </c>
+      <c r="F91">
+        <v>7.0507248586712796</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>97</v>
+      </c>
+      <c r="B93">
+        <v>6.3510278151136701</v>
+      </c>
+      <c r="C93">
+        <v>6.3506465779538903</v>
+      </c>
+      <c r="D93">
+        <v>6.2234404863337902</v>
+      </c>
+      <c r="E93">
+        <v>6.3526798421438899</v>
+      </c>
+      <c r="F93">
+        <v>6.2280153308064197</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>98</v>
+      </c>
+      <c r="B94">
+        <v>5.8906205522364701</v>
+      </c>
+      <c r="C94">
+        <v>5.8885872880239098</v>
+      </c>
+      <c r="D94">
+        <v>5.8315288113649002</v>
+      </c>
+      <c r="E94">
+        <v>5.7610558741045104</v>
+      </c>
+      <c r="F94">
+        <v>5.8287330730585101</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>103</v>
+      </c>
+      <c r="B99">
+        <v>9.0499318845433905</v>
+      </c>
+      <c r="C99">
+        <v>9.05908157493338</v>
+      </c>
+      <c r="D99">
+        <v>8.9140844220571598</v>
+      </c>
+      <c r="E99">
+        <v>9.0871660357999993</v>
+      </c>
+      <c r="F99">
+        <v>8.9419147247885995</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>106</v>
+      </c>
+      <c r="B102">
+        <v>6.9372433006496603</v>
+      </c>
+      <c r="C102">
+        <v>6.6450886503296402</v>
+      </c>
+      <c r="D102">
+        <v>6.45586800064385</v>
+      </c>
+      <c r="E102">
+        <v>6.4198919319408398</v>
+      </c>
+      <c r="F102">
+        <v>6.4722611932772596</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>107</v>
+      </c>
+      <c r="B103">
+        <v>0.25441218324021198</v>
+      </c>
+      <c r="C103">
+        <v>0.25441218324021198</v>
+      </c>
+      <c r="D103">
+        <v>0.124791590450923</v>
+      </c>
+      <c r="E103">
+        <v>0.25098104999999998</v>
+      </c>
+      <c r="F103">
+        <v>0.14054938787822399</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>109</v>
+      </c>
+      <c r="B105">
+        <v>0.80263104346948</v>
+      </c>
+      <c r="C105">
+        <v>0.80377475549058897</v>
+      </c>
+      <c r="D105">
+        <v>1.15883351532281</v>
+      </c>
+      <c r="E105">
+        <v>0.79958114763596499</v>
+      </c>
+      <c r="F105">
+        <v>1.16137509614722</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>111</v>
+      </c>
+      <c r="B107">
+        <v>0.19786202253840701</v>
+      </c>
+      <c r="C107">
+        <v>0.19887865472369901</v>
+      </c>
+      <c r="D107">
+        <v>0.119073035040723</v>
+      </c>
+      <c r="E107">
+        <v>0.20243686701103999</v>
+      </c>
+      <c r="F107">
+        <v>0.116785612804406</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>113</v>
+      </c>
+      <c r="B109">
+        <v>1.56688422591718</v>
+      </c>
+      <c r="C109">
+        <v>1.56548635684299</v>
+      </c>
+      <c r="D109">
+        <v>1.53473323567588</v>
+      </c>
+      <c r="E109">
+        <v>1.565740514</v>
+      </c>
+      <c r="F109">
+        <v>1.53244581343957</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>114</v>
+      </c>
+      <c r="B110">
+        <v>1.83006486112346</v>
+      </c>
+      <c r="C110">
+        <v>1.8276503598639899</v>
+      </c>
+      <c r="D110">
+        <v>1.78101236224642</v>
+      </c>
+      <c r="E110">
+        <v>1.8276503599</v>
+      </c>
+      <c r="F110">
+        <v>1.77885201903326</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>118</v>
+      </c>
+      <c r="B114">
+        <v>1.57425480862848</v>
+      </c>
+      <c r="C114">
+        <v>1.5715861494129699</v>
+      </c>
+      <c r="D114">
+        <v>1.5217711763969499</v>
+      </c>
+      <c r="E114">
+        <v>1.5717132283449999</v>
+      </c>
+      <c r="F114">
+        <v>1.5201191492764401</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>121</v>
+      </c>
+      <c r="B117">
+        <v>5.5003609043203703</v>
+      </c>
+      <c r="C117">
+        <v>5.4978193242183204</v>
+      </c>
+      <c r="D117">
+        <v>5.35180553879563</v>
+      </c>
+      <c r="E117">
+        <v>5.3676230635218296</v>
+      </c>
+      <c r="F117">
+        <v>5.3532034079601098</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>123</v>
+      </c>
+      <c r="B119">
+        <v>0.51555955407591703</v>
+      </c>
+      <c r="C119">
+        <v>0.51454292225180598</v>
+      </c>
+      <c r="D119">
+        <v>0.318968321588534</v>
+      </c>
+      <c r="E119">
+        <v>0.51390752740688395</v>
+      </c>
+      <c r="F119">
+        <v>0.31833292674361202</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>125</v>
+      </c>
+      <c r="B121">
+        <v>3.1567697529498</v>
+      </c>
+      <c r="C121">
+        <v>3.15651559544524</v>
+      </c>
+      <c r="D121">
+        <v>2.8635984708056599</v>
+      </c>
+      <c r="E121">
+        <v>3.1446972472799999</v>
+      </c>
+      <c r="F121">
+        <v>2.85127180691343</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>127</v>
+      </c>
+      <c r="B123">
+        <v>0.72651071554848101</v>
+      </c>
+      <c r="C123">
+        <v>0.72562116211546601</v>
+      </c>
+      <c r="D123">
+        <v>0.63285348297296995</v>
+      </c>
+      <c r="E123">
+        <v>0.72651071509999998</v>
+      </c>
+      <c r="F123">
+        <v>0.634759668230097</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
+        <v>129</v>
+      </c>
+      <c r="B125">
+        <v>0.64784880608071205</v>
+      </c>
+      <c r="C125">
+        <v>0.64797588519416804</v>
+      </c>
+      <c r="D125">
+        <v>0.58469053725805198</v>
+      </c>
+      <c r="E125">
+        <v>0.64759464919999998</v>
+      </c>
+      <c r="F125">
+        <v>0.58710503896900501</v>
+      </c>
+    </row>
+    <row r="126" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A126" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="127" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A127" t="s">
+        <v>131</v>
+      </c>
+      <c r="B127">
+        <v>0.38288906545311402</v>
+      </c>
+      <c r="C127">
+        <v>0.383524460298036</v>
+      </c>
+      <c r="D127">
+        <v>0.314774714095091</v>
+      </c>
+      <c r="E127">
+        <v>0.38682851434999999</v>
+      </c>
+      <c r="F127">
+        <v>0.31769753153750901</v>
+      </c>
+    </row>
+    <row r="128" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A128" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="129" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A129" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="130" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A130" t="s">
+        <v>134</v>
+      </c>
+      <c r="B130">
+        <v>0.74836830536517196</v>
+      </c>
+      <c r="C130">
+        <v>0.74862246359208495</v>
+      </c>
+      <c r="D130">
+        <v>0.57185555691198897</v>
+      </c>
+      <c r="E130">
+        <v>0.75319730878707802</v>
+      </c>
+      <c r="F130">
+        <v>0.56905981786066695</v>
+      </c>
+    </row>
+    <row r="131" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A131" t="s">
+        <v>135</v>
+      </c>
+      <c r="B131">
+        <v>0.93504737494891199</v>
+      </c>
+      <c r="C131">
+        <v>0.93695356020603904</v>
+      </c>
+      <c r="D131">
+        <v>0.76704892059607199</v>
+      </c>
+      <c r="E131">
+        <v>0.93352242703215405</v>
+      </c>
+      <c r="F131">
+        <v>0.76171160216506095</v>
+      </c>
+    </row>
+    <row r="132" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A132" t="s">
+        <v>136</v>
+      </c>
+      <c r="B132">
+        <v>0.42304603352151499</v>
+      </c>
+      <c r="C132">
+        <v>0.422410637954232</v>
+      </c>
+      <c r="D132">
+        <v>0.39750315122048602</v>
+      </c>
+      <c r="E132">
+        <v>0.42838335123010002</v>
+      </c>
+      <c r="F132">
+        <v>0.40004473132253499</v>
+      </c>
+    </row>
+    <row r="133" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A133" t="s">
+        <v>137</v>
+      </c>
+      <c r="B133">
+        <v>0.52165934682648796</v>
+      </c>
+      <c r="C133">
+        <v>0.52115103037266097</v>
+      </c>
+      <c r="D133">
+        <v>0.49662478170164498</v>
+      </c>
+      <c r="E133">
+        <v>0.528902851236</v>
+      </c>
+      <c r="F133">
+        <v>0.49942051930824699</v>
+      </c>
+    </row>
+    <row r="134" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A134" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="135" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A135" t="s">
+        <v>139</v>
+      </c>
+      <c r="B135">
+        <v>0.56651823848097804</v>
+      </c>
+      <c r="C135">
+        <v>0.56651823848097804</v>
+      </c>
+      <c r="D135">
+        <v>0.54923549277573902</v>
+      </c>
+      <c r="E135">
+        <v>0.57503253185799996</v>
+      </c>
+      <c r="F135">
+        <v>0.55215831021815798</v>
+      </c>
+    </row>
+    <row r="136" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A136" t="s">
+        <v>140</v>
+      </c>
+      <c r="B136">
+        <v>4.0034972141153897</v>
+      </c>
+      <c r="C136">
+        <v>4.0027347401570097</v>
+      </c>
+      <c r="D136">
+        <v>3.7018116378709101</v>
+      </c>
+      <c r="E136">
+        <v>4.0060387949390002</v>
+      </c>
+      <c r="F136">
+        <v>3.6996512951092302</v>
+      </c>
+    </row>
+    <row r="137" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A137" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="138" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A138" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="139" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A139" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="140" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A140" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="141" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A141" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="142" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A142" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="143" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A143" t="s">
+        <v>147</v>
+      </c>
+      <c r="B143">
+        <v>0.46510918829176401</v>
+      </c>
+      <c r="C143">
+        <v>0.46155097600442402</v>
+      </c>
+      <c r="D143">
+        <v>0.39940933431053099</v>
+      </c>
+      <c r="E143">
+        <v>0.46739660655499998</v>
+      </c>
+      <c r="F143">
+        <v>0.40258631359166602</v>
+      </c>
+    </row>
+    <row r="144" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A144" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="145" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A145" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="146" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A146" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="147" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A147" t="s">
+        <v>151</v>
+      </c>
+      <c r="B147">
+        <v>0.99998475063760295</v>
+      </c>
+      <c r="C147">
+        <v>0.972544579672035</v>
+      </c>
+      <c r="D147">
+        <v>0.967198364648436</v>
+      </c>
+      <c r="E147">
+        <v>1.0097698344199999</v>
+      </c>
+      <c r="F147">
+        <v>0.972154446461438</v>
+      </c>
+    </row>
+    <row r="148" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A148" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="149" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A149" t="s">
+        <v>153</v>
+      </c>
+      <c r="B149">
+        <v>1.3720721001152301</v>
+      </c>
+      <c r="C149">
+        <v>1.3725804151243399</v>
+      </c>
+      <c r="D149">
+        <v>1.3128532794755601</v>
+      </c>
+      <c r="E149">
+        <v>1.3856695536900001</v>
+      </c>
+      <c r="F149">
+        <v>1.31717396499892</v>
+      </c>
+    </row>
+    <row r="150" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A150" t="s">
+        <v>154</v>
+      </c>
+      <c r="B150">
+        <v>1.34462303255708</v>
+      </c>
+      <c r="C150">
+        <v>1.34411471682561</v>
+      </c>
+      <c r="D150">
+        <v>1.2554135657019201</v>
+      </c>
+      <c r="E150">
+        <v>1.35186653624522</v>
+      </c>
+      <c r="F150">
+        <v>1.25897177798926</v>
+      </c>
+    </row>
+    <row r="151" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A151" t="s">
+        <v>155</v>
+      </c>
+      <c r="B151">
+        <v>3.57562217861669</v>
+      </c>
+      <c r="C151">
+        <v>3.5756221793390499</v>
+      </c>
+      <c r="D151">
+        <v>3.1472388273865199</v>
+      </c>
+      <c r="E151">
+        <v>3.5643121461873801</v>
+      </c>
+      <c r="F151">
+        <v>3.1317351878249502</v>
+      </c>
+    </row>
+    <row r="152" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A152" t="s">
+        <v>156</v>
+      </c>
+      <c r="B152">
+        <v>1.8764487012364801</v>
+      </c>
+      <c r="C152">
+        <v>1.8760674638961099</v>
+      </c>
+      <c r="D152">
+        <v>1.6275009144571999</v>
+      </c>
+      <c r="E152">
+        <v>1.87899028061617</v>
+      </c>
+      <c r="F152">
+        <v>1.63258407610602</v>
+      </c>
+    </row>
+    <row r="153" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A153" t="s">
+        <v>157</v>
+      </c>
+      <c r="B153">
+        <v>1.8326064410449201</v>
+      </c>
+      <c r="C153">
+        <v>1.8328605992718401</v>
+      </c>
+      <c r="D153">
+        <v>1.5435016876419601</v>
+      </c>
+      <c r="E153">
+        <v>1.8244733842848999</v>
+      </c>
+      <c r="F153">
+        <v>1.5391810013962399</v>
+      </c>
+    </row>
+    <row r="154" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A154" t="s">
+        <v>187</v>
+      </c>
+      <c r="B154">
+        <v>4.3206863901915998E-2</v>
+      </c>
+      <c r="C154">
+        <v>4.0919442026780002E-2</v>
+      </c>
+      <c r="D154">
+        <v>5.8075109340922602E-2</v>
+      </c>
+      <c r="E154">
+        <v>3.8123703697817903E-2</v>
+      </c>
+      <c r="F154">
+        <v>5.6041844970339101E-2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0606D0F1-59E7-40AC-A041-B0BE0EF69D62}">
   <dimension ref="A1:C72"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -8624,7 +10505,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B22EC2D2-A040-470E-AC95-ACA37FA2C4F6}">
   <dimension ref="A1:C72"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -9426,7 +11307,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31844E60-7C27-4306-8B91-39464BD49E59}">
   <dimension ref="A1:C72"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -10230,7 +12111,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F16AC4A-06F6-4838-A630-E168C701BFF7}">
-  <dimension ref="A1:M154"/>
+  <dimension ref="A1:M155"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
@@ -15640,14 +17521,47 @@
         <v>1.0562</v>
       </c>
     </row>
+    <row r="155" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A155" t="s">
+        <v>187</v>
+      </c>
+      <c r="B155">
+        <v>5.7000000000000002E-3</v>
+      </c>
+      <c r="F155">
+        <v>5.8999999999999999E-3</v>
+      </c>
+      <c r="G155">
+        <v>4.32068646242766E-2</v>
+      </c>
+      <c r="H155">
+        <v>3.6598755781060498E-2</v>
+      </c>
+      <c r="I155">
+        <v>3.8250782811274399E-2</v>
+      </c>
+      <c r="J155">
+        <v>2.8999999999999998E-3</v>
+      </c>
+      <c r="K155">
+        <v>4.4858891654490501E-2</v>
+      </c>
+      <c r="L155">
+        <v>3.8250782811274399E-2</v>
+      </c>
+      <c r="M155">
+        <v>3.95215725011187E-2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FAD3F1BA-E3FB-4E66-AD27-2E9ECE39DF41}">
-  <dimension ref="A1:G153"/>
+  <dimension ref="A1:G154"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -19167,6 +21081,26 @@
       </c>
       <c r="G153">
         <v>1.4478</v>
+      </c>
+    </row>
+    <row r="154" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A154" t="s">
+        <v>187</v>
+      </c>
+      <c r="B154">
+        <v>4.24E-2</v>
+      </c>
+      <c r="C154">
+        <v>4.2200000000000001E-2</v>
+      </c>
+      <c r="D154">
+        <v>6.6716481832361604E-2</v>
+      </c>
+      <c r="E154">
+        <v>4.0399999999999998E-2</v>
+      </c>
+      <c r="F154">
+        <v>6.5954007873982895E-2</v>
       </c>
     </row>
   </sheetData>
@@ -19176,7 +21110,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2458C5C3-EFC5-48BD-91B0-1ED54F173F9F}">
-  <dimension ref="A1:G153"/>
+  <dimension ref="A1:G154"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -22696,6 +24630,26 @@
       </c>
       <c r="G153">
         <v>1.4487000000000001</v>
+      </c>
+    </row>
+    <row r="154" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A154" t="s">
+        <v>187</v>
+      </c>
+      <c r="B154">
+        <v>3.1199999999999999E-2</v>
+      </c>
+      <c r="C154">
+        <v>3.1E-2</v>
+      </c>
+      <c r="D154">
+        <v>6.1379163401350301E-2</v>
+      </c>
+      <c r="E154">
+        <v>2.9100000000000001E-2</v>
+      </c>
+      <c r="F154">
+        <v>6.0870846947524197E-2</v>
       </c>
     </row>
   </sheetData>
@@ -22705,7 +24659,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82A83B5F-5585-4182-88EC-A36770133EBC}">
-  <dimension ref="A1:G153"/>
+  <dimension ref="A1:G154"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -26225,6 +28179,26 @@
       </c>
       <c r="G153">
         <v>1.4816</v>
+      </c>
+    </row>
+    <row r="154" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A154" t="s">
+        <v>187</v>
+      </c>
+      <c r="B154">
+        <v>1.7500000000000002E-2</v>
+      </c>
+      <c r="C154">
+        <v>1.7600000000000001E-2</v>
+      </c>
+      <c r="D154">
+        <v>2.77032250627085E-2</v>
+      </c>
+      <c r="E154">
+        <v>1.37E-2</v>
+      </c>
+      <c r="F154">
+        <v>2.6051198032494598E-2</v>
       </c>
     </row>
   </sheetData>
@@ -26234,7 +28208,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD369F19-41E3-4974-BE37-1FC579F300E4}">
-  <dimension ref="A1:G153"/>
+  <dimension ref="A1:G154"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.5703125" bestFit="1" customWidth="1"/>
@@ -29757,6 +31731,26 @@
       </c>
       <c r="G153">
         <v>1.4424999999999999</v>
+      </c>
+    </row>
+    <row r="154" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A154" t="s">
+        <v>187</v>
+      </c>
+      <c r="B154">
+        <v>4.1999999999999997E-3</v>
+      </c>
+      <c r="C154">
+        <v>4.3E-3</v>
+      </c>
+      <c r="D154">
+        <v>2.0968037106035901E-2</v>
+      </c>
+      <c r="E154">
+        <v>6.1000000000000004E-3</v>
+      </c>
+      <c r="F154">
+        <v>2.1476353559862001E-2</v>
       </c>
     </row>
   </sheetData>
@@ -33295,7 +35289,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9247ECA6-2E05-4FC5-B207-880784AF6FCE}">
-  <dimension ref="A1:G153"/>
+  <dimension ref="A1:G154"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -36817,14 +38811,35 @@
         <v>1.5225</v>
       </c>
     </row>
+    <row r="154" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A154" t="s">
+        <v>187</v>
+      </c>
+      <c r="B154">
+        <v>4.2500000000000003E-2</v>
+      </c>
+      <c r="C154">
+        <v>4.2799999999999998E-2</v>
+      </c>
+      <c r="D154">
+        <v>5.2356553569541699E-2</v>
+      </c>
+      <c r="E154">
+        <v>4.1399999999999999E-2</v>
+      </c>
+      <c r="F154">
+        <v>5.2102395342628602E-2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{96217BAD-7789-496E-9FEF-757FEDCE6C9D}">
-  <dimension ref="A1:G153"/>
+  <dimension ref="A1:G154"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -40346,6 +42361,26 @@
         <v>1.5296000000000001</v>
       </c>
     </row>
+    <row r="154" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A154" t="s">
+        <v>187</v>
+      </c>
+      <c r="B154">
+        <v>3.18968321949714E-2</v>
+      </c>
+      <c r="C154">
+        <v>3.1642673968058303E-2</v>
+      </c>
+      <c r="D154">
+        <v>5.3266438923902502E-2</v>
+      </c>
+      <c r="E154">
+        <v>2.96094103198354E-2</v>
+      </c>
+      <c r="F154">
+        <v>5.2331138035794603E-2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>